<commit_message>
Rediseño de dashboards, importación Excel en drawer y roles GERENCIA e IT
</commit_message>
<xml_diff>
--- a/docs/ejemplos-importacion/creditos.xlsx
+++ b/docs/ejemplos-importacion/creditos.xlsx
@@ -1,42 +1,161 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30527"/>
   <workbookPr codeName="ThisWorkbook"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Dell\Desktop\Comisariato Web\sistema-comisariato-web\docs\ejemplos-importacion\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{38D8C94F-87F2-47CC-86C3-482A75081A7F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <bookViews>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+  </bookViews>
   <sheets>
     <sheet name="creditos" sheetId="1" r:id="rId1"/>
   </sheets>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
-<file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
-<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
-  <metadataTypes count="1">
-    <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
-  </metadataTypes>
-  <futureMetadata name="XLDAPR" count="1">
-    <bk>
-      <extLst>
-        <ext uri="{bdbb8cdc-fa1e-496e-a857-3c3f30c029c3}">
-          <xda:dynamicArrayProperties fDynamic="1" fCollapsed="0"/>
-        </ext>
-      </extLst>
-    </bk>
-  </futureMetadata>
-  <cellMetadata count="1">
-    <bk>
-      <rc t="1" v="0"/>
-    </bk>
-  </cellMetadata>
-</metadata>
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="40">
+  <si>
+    <t>creditoId</t>
+  </si>
+  <si>
+    <t>empleadoId</t>
+  </si>
+  <si>
+    <t>productoId</t>
+  </si>
+  <si>
+    <t>cantidad</t>
+  </si>
+  <si>
+    <t>plazoMeses</t>
+  </si>
+  <si>
+    <t>cuotaMensual</t>
+  </si>
+  <si>
+    <t>totalCredito</t>
+  </si>
+  <si>
+    <t>cuotasPagadas</t>
+  </si>
+  <si>
+    <t>estado</t>
+  </si>
+  <si>
+    <t>fechaSolicitud</t>
+  </si>
+  <si>
+    <t>fechaResolucion</t>
+  </si>
+  <si>
+    <t>CRD-H01</t>
+  </si>
+  <si>
+    <t>Aprobado</t>
+  </si>
+  <si>
+    <t>CRD-H02</t>
+  </si>
+  <si>
+    <t>2026-02-05</t>
+  </si>
+  <si>
+    <t>2026-02-07</t>
+  </si>
+  <si>
+    <t>CRD-H03</t>
+  </si>
+  <si>
+    <t>EMP-005</t>
+  </si>
+  <si>
+    <t>18/06/2026</t>
+  </si>
+  <si>
+    <t>20/06/2026</t>
+  </si>
+  <si>
+    <t>CRD-H04</t>
+  </si>
+  <si>
+    <t>EMP-007</t>
+  </si>
+  <si>
+    <t>Rechazado</t>
+  </si>
+  <si>
+    <t>CRD-H05</t>
+  </si>
+  <si>
+    <t>CRD-H06</t>
+  </si>
+  <si>
+    <t>CRD-H07</t>
+  </si>
+  <si>
+    <t>EMP-006</t>
+  </si>
+  <si>
+    <t>CRD-001</t>
+  </si>
+  <si>
+    <t>Pendiente</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t>EMP-010</t>
+  </si>
+  <si>
+    <t>EMP-009</t>
+  </si>
+  <si>
+    <t>EMP-008</t>
+  </si>
+  <si>
+    <t>EMP-011</t>
+  </si>
+  <si>
+    <t>EMP-012</t>
+  </si>
+  <si>
+    <t>PROD-001</t>
+  </si>
+  <si>
+    <t>PROD-002</t>
+  </si>
+  <si>
+    <t>PROD-004</t>
+  </si>
+  <si>
+    <t>PROD-016</t>
+  </si>
+  <si>
+    <t>PROD-005</t>
+  </si>
+</sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:vt="http://schemas.openxmlformats.org/officeDocument/2006/docPropsVTypes">
-  <numFmts count="1">
-    <numFmt numFmtId="56" formatCode="&quot;上午/下午 &quot;hh&quot;時&quot;mm&quot;分&quot;ss&quot;秒 &quot;"/>
-  </numFmts>
-  <fonts count="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
       <sz val="12"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -64,15 +183,24 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+  <cellXfs count="3">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleMedium4"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
@@ -397,53 +525,54 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:K9"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:K15"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1">
-      <c r="A1" t="str">
-        <v>creditoId</v>
-      </c>
-      <c r="B1" t="str">
-        <v>empleadoId</v>
-      </c>
-      <c r="C1" t="str">
-        <v>productoId</v>
-      </c>
-      <c r="D1" t="str">
-        <v>cantidad</v>
-      </c>
-      <c r="E1" t="str">
-        <v>plazoMeses</v>
-      </c>
-      <c r="F1" t="str">
-        <v>cuotaMensual</v>
-      </c>
-      <c r="G1" t="str">
-        <v>totalCredito</v>
-      </c>
-      <c r="H1" t="str">
-        <v>cuotasPagadas</v>
-      </c>
-      <c r="I1" t="str">
-        <v>estado</v>
-      </c>
-      <c r="J1" t="str">
-        <v>fechaSolicitud</v>
-      </c>
-      <c r="K1" t="str">
-        <v>fechaResolucion</v>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="str">
-        <v>CRD-H01</v>
-      </c>
-      <c r="B2" t="str">
-        <v>EMP-002</v>
-      </c>
-      <c r="C2" t="str">
-        <v>PRD-001</v>
+    <row r="1" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" t="s">
+        <v>9</v>
+      </c>
+      <c r="K1" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="2" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>11</v>
+      </c>
+      <c r="B2" t="s">
+        <v>30</v>
+      </c>
+      <c r="C2" t="s">
+        <v>35</v>
       </c>
       <c r="D2">
         <v>1</v>
@@ -460,25 +589,25 @@
       <c r="H2">
         <v>4</v>
       </c>
-      <c r="I2" t="str">
-        <v>Aprobado</v>
-      </c>
-      <c r="J2" s="1" t="d">
-        <v>2026-03-10T12:00:00.000Z</v>
-      </c>
-      <c r="K2" s="1" t="d">
-        <v>2026-03-12T12:00:00.000Z</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="str">
-        <v>CRD-H02</v>
-      </c>
-      <c r="B3" t="str">
-        <v>EMP-004</v>
-      </c>
-      <c r="C3" t="str">
-        <v>PRD-002</v>
+      <c r="I2" t="s">
+        <v>12</v>
+      </c>
+      <c r="J2" s="1">
+        <v>46091.5</v>
+      </c>
+      <c r="K2" s="1">
+        <v>46093.5</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>13</v>
+      </c>
+      <c r="B3" t="s">
+        <v>31</v>
+      </c>
+      <c r="C3" t="s">
+        <v>36</v>
       </c>
       <c r="D3">
         <v>2</v>
@@ -495,25 +624,25 @@
       <c r="H3">
         <v>3</v>
       </c>
-      <c r="I3" t="str">
-        <v>Aprobado</v>
-      </c>
-      <c r="J3" t="str">
-        <v>2026-02-05</v>
-      </c>
-      <c r="K3" t="str">
-        <v>2026-02-07</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="str">
-        <v>CRD-H03</v>
-      </c>
-      <c r="B4" t="str">
-        <v>EMP-005</v>
-      </c>
-      <c r="C4" t="str">
-        <v>PRD-003</v>
+      <c r="I3" t="s">
+        <v>12</v>
+      </c>
+      <c r="J3" t="s">
+        <v>14</v>
+      </c>
+      <c r="K3" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>16</v>
+      </c>
+      <c r="B4" t="s">
+        <v>17</v>
+      </c>
+      <c r="C4" t="s">
+        <v>39</v>
       </c>
       <c r="D4">
         <v>1</v>
@@ -530,25 +659,25 @@
       <c r="H4">
         <v>2</v>
       </c>
-      <c r="I4" t="str">
-        <v>Aprobado</v>
-      </c>
-      <c r="J4" t="str">
-        <v>18/06/2026</v>
-      </c>
-      <c r="K4" t="str">
-        <v>20/06/2026</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="str">
-        <v>CRD-H04</v>
-      </c>
-      <c r="B5" t="str">
-        <v>EMP-007</v>
-      </c>
-      <c r="C5" t="str">
-        <v>PRD-004</v>
+      <c r="I4" t="s">
+        <v>12</v>
+      </c>
+      <c r="J4" t="s">
+        <v>18</v>
+      </c>
+      <c r="K4" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>20</v>
+      </c>
+      <c r="B5" t="s">
+        <v>21</v>
+      </c>
+      <c r="C5" t="s">
+        <v>37</v>
       </c>
       <c r="D5">
         <v>1</v>
@@ -565,25 +694,25 @@
       <c r="H5">
         <v>0</v>
       </c>
-      <c r="I5" t="str">
-        <v>Rechazado</v>
-      </c>
-      <c r="J5" s="1" t="d">
-        <v>2026-08-01T12:00:00.000Z</v>
-      </c>
-      <c r="K5" s="1" t="d">
-        <v>2026-08-03T12:00:00.000Z</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="str">
-        <v>CRD-H05</v>
-      </c>
-      <c r="B6" t="str">
-        <v>EMP-003</v>
-      </c>
-      <c r="C6" t="str">
-        <v>PRD-002</v>
+      <c r="I5" t="s">
+        <v>22</v>
+      </c>
+      <c r="J5" s="1">
+        <v>46235.5</v>
+      </c>
+      <c r="K5" s="1">
+        <v>46237.5</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>23</v>
+      </c>
+      <c r="B6" t="s">
+        <v>32</v>
+      </c>
+      <c r="C6" t="s">
+        <v>36</v>
       </c>
       <c r="D6">
         <v>1</v>
@@ -600,25 +729,25 @@
       <c r="H6">
         <v>1</v>
       </c>
-      <c r="I6" t="str">
-        <v>Aprobado</v>
-      </c>
-      <c r="J6" s="1" t="d">
-        <v>2026-09-02T12:00:00.000Z</v>
-      </c>
-      <c r="K6" s="1" t="d">
-        <v>2026-09-04T12:00:00.000Z</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="str">
-        <v>CRD-H06</v>
-      </c>
-      <c r="B7" t="str">
-        <v>EMP-002</v>
-      </c>
-      <c r="C7" t="str">
-        <v>PRD-777</v>
+      <c r="I6" t="s">
+        <v>12</v>
+      </c>
+      <c r="J6" s="1">
+        <v>46267.5</v>
+      </c>
+      <c r="K6" s="1">
+        <v>46269.5</v>
+      </c>
+    </row>
+    <row r="7" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
+        <v>24</v>
+      </c>
+      <c r="B7" t="s">
+        <v>33</v>
+      </c>
+      <c r="C7" t="s">
+        <v>38</v>
       </c>
       <c r="D7">
         <v>1</v>
@@ -635,25 +764,25 @@
       <c r="H7">
         <v>0</v>
       </c>
-      <c r="I7" t="str">
-        <v>Aprobado</v>
-      </c>
-      <c r="J7" s="1" t="d">
-        <v>2026-04-01T12:00:00.000Z</v>
-      </c>
-      <c r="K7" s="1" t="d">
-        <v>2026-04-02T12:00:00.000Z</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="str">
-        <v>CRD-H07</v>
-      </c>
-      <c r="B8" t="str">
-        <v>EMP-006</v>
-      </c>
-      <c r="C8" t="str">
-        <v>PRD-001</v>
+      <c r="I7" t="s">
+        <v>12</v>
+      </c>
+      <c r="J7" s="1">
+        <v>46113.5</v>
+      </c>
+      <c r="K7" s="1">
+        <v>46114.5</v>
+      </c>
+    </row>
+    <row r="8" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A8" t="s">
+        <v>25</v>
+      </c>
+      <c r="B8" t="s">
+        <v>26</v>
+      </c>
+      <c r="C8" t="s">
+        <v>35</v>
       </c>
       <c r="D8">
         <v>1</v>
@@ -668,27 +797,27 @@
         <v>9804</v>
       </c>
       <c r="H8">
-        <v>15</v>
-      </c>
-      <c r="I8" t="str">
-        <v>Aprobado</v>
-      </c>
-      <c r="J8" s="1" t="d">
-        <v>2026-04-01T12:00:00.000Z</v>
-      </c>
-      <c r="K8" s="1" t="d">
-        <v>2026-04-02T12:00:00.000Z</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="str">
-        <v>CRD-001</v>
-      </c>
-      <c r="B9" t="str">
-        <v>EMP-002</v>
-      </c>
-      <c r="C9" t="str">
-        <v>PRD-002</v>
+        <v>8</v>
+      </c>
+      <c r="I8" t="s">
+        <v>12</v>
+      </c>
+      <c r="J8" s="1">
+        <v>46113.5</v>
+      </c>
+      <c r="K8" s="1">
+        <v>46114.5</v>
+      </c>
+    </row>
+    <row r="9" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A9" t="s">
+        <v>27</v>
+      </c>
+      <c r="B9" t="s">
+        <v>34</v>
+      </c>
+      <c r="C9" t="s">
+        <v>36</v>
       </c>
       <c r="D9">
         <v>2</v>
@@ -705,19 +834,26 @@
       <c r="H9">
         <v>0</v>
       </c>
-      <c r="I9" t="str">
-        <v>Pendiente</v>
-      </c>
-      <c r="J9" s="1" t="d">
-        <v>2026-10-01T12:00:00.000Z</v>
-      </c>
-      <c r="K9" t="str">
-        <v/>
-      </c>
+      <c r="I9" t="s">
+        <v>28</v>
+      </c>
+      <c r="J9" s="1">
+        <v>46296.5</v>
+      </c>
+      <c r="K9" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="13" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="F13" s="2"/>
+    </row>
+    <row r="15" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="E15" s="2"/>
     </row>
   </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:K9"/>
+    <ignoredError sqref="A1:K1 A5:B5 A2 D2:K2 A3 D3:K3 A8:B8 A6 D6:K6 A7 D7:K7 A9 D9:K9 A4:B4 D4:K4 D5:K5 D8:G8 I8:K8" numberStoredAsText="1"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>